<commit_message>
Add radar and FFS ground heights to Excel and scenario exports
</commit_message>
<xml_diff>
--- a/data/HSS/air_defense_master.xlsx
+++ b/data/HSS/air_defense_master.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="master" sheetId="1" r:id="R52ce37eb5e274b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="munition_costs" sheetId="2" r:id="R7bd5567e86444539"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="master" sheetId="1" r:id="Rf6c50a8343ca4e53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="munition_costs" sheetId="2" r:id="Rdf64627404bb4538"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,8 +14,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="3">
     <x:numFmt numFmtId="200" formatCode="#,##0&quot; USD&quot;"/>
+    <x:numFmt numFmtId="201" formatCode="0.##&quot; m&quot;"/>
+    <x:numFmt numFmtId="202" formatCode="0&quot; m&quot;"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -57,7 +59,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="7">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -71,6 +73,8 @@
       </x:extLst>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -292,6 +296,8 @@
   <x:cols>
     <x:col min="44" max="44" width="24" hidden="0" customWidth="1"/>
     <x:col min="45" max="45" width="24" hidden="0" customWidth="1"/>
+    <x:col min="46" max="46" width="36" hidden="0" customWidth="1"/>
+    <x:col min="47" max="47" width="36" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -516,6 +522,12 @@
       <x:c r="AS1" s="6" t="str">
         <x:v>FSS_LOS_needed</x:v>
       </x:c>
+      <x:c r="AT1" s="6" t="str">
+        <x:v>radar_height_above_ground_m</x:v>
+      </x:c>
+      <x:c r="AU1" s="6" t="str">
+        <x:v>ffs_height_above_ground_m</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="inlineStr">
@@ -663,6 +675,12 @@
       <x:c r="AS2" s="5" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AT2" s="7" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="AU2" s="8" t="n">
+        <x:v>2</x:v>
+      </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="inlineStr">
@@ -810,6 +828,12 @@
       <x:c r="AS3" s="5" t="b">
         <x:v>1</x:v>
       </x:c>
+      <x:c r="AT3" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="AU3" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="inlineStr">
@@ -957,6 +981,12 @@
       <x:c r="AS4" s="5" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AT4" s="7" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="AU4" s="8" t="n">
+        <x:v>3</x:v>
+      </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="inlineStr">
@@ -1104,6 +1134,12 @@
       <x:c r="AS5" s="5" t="b">
         <x:v>0</x:v>
       </x:c>
+      <x:c r="AT5" s="7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="AU5" s="8" t="n">
+        <x:v>4</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="inlineStr">
@@ -1250,6 +1286,12 @@
       </x:c>
       <x:c r="AS6" s="5" t="b">
         <x:v>0</x:v>
+      </x:c>
+      <x:c r="AT6" s="7" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="AU6" s="8" t="n">
+        <x:v>4</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add editable radar RCS bounds to Excel and JSON exports
</commit_message>
<xml_diff>
--- a/data/HSS/air_defense_master.xlsx
+++ b/data/HSS/air_defense_master.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="master" sheetId="1" r:id="Rf6c50a8343ca4e53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="munition_costs" sheetId="2" r:id="Rdf64627404bb4538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="master" sheetId="1" r:id="Rf75884b5373b4e7f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="munition_costs" sheetId="2" r:id="R68e827c2ae964110"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,10 +14,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="4">
     <x:numFmt numFmtId="200" formatCode="#,##0&quot; USD&quot;"/>
     <x:numFmt numFmtId="201" formatCode="0.##&quot; m&quot;"/>
     <x:numFmt numFmtId="202" formatCode="0&quot; m&quot;"/>
+    <x:numFmt numFmtId="203" formatCode="0.00&quot; m²&quot;"/>
   </x:numFmts>
   <x:fonts count="4">
     <x:font>
@@ -59,7 +60,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="9">
+  <x:cellXfs count="10">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -75,6 +76,7 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="202" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -298,6 +300,10 @@
     <x:col min="45" max="45" width="24" hidden="0" customWidth="1"/>
     <x:col min="46" max="46" width="36" hidden="0" customWidth="1"/>
     <x:col min="47" max="47" width="36" hidden="0" customWidth="1"/>
+    <x:col min="48" max="48" width="24" hidden="0" customWidth="1"/>
+    <x:col min="49" max="49" width="24" hidden="0" customWidth="1"/>
+    <x:col min="50" max="50" width="24" hidden="0" customWidth="1"/>
+    <x:col min="51" max="51" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -528,6 +534,18 @@
       <x:c r="AU1" s="6" t="str">
         <x:v>ffs_height_above_ground_m</x:v>
       </x:c>
+      <x:c r="AV1" s="6" t="str">
+        <x:v>radar_min_rcs_m2</x:v>
+      </x:c>
+      <x:c r="AW1" s="6" t="str">
+        <x:v>radar_max_rcs_m2</x:v>
+      </x:c>
+      <x:c r="AX1" s="6" t="str">
+        <x:v>akr_min_rcs_m2</x:v>
+      </x:c>
+      <x:c r="AY1" s="6" t="str">
+        <x:v>akr_max_rcs_m2</x:v>
+      </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="inlineStr">
@@ -681,6 +699,14 @@
       <x:c r="AU2" s="8" t="n">
         <x:v>2</x:v>
       </x:c>
+      <x:c r="AV2" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW2" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AX2" s="9"/>
+      <x:c r="AY2" s="9"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="inlineStr">
@@ -834,6 +860,14 @@
       <x:c r="AU3" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="AV3" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW3" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AX3" s="9"/>
+      <x:c r="AY3" s="9"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="inlineStr">
@@ -987,6 +1021,14 @@
       <x:c r="AU4" s="8" t="n">
         <x:v>3</x:v>
       </x:c>
+      <x:c r="AV4" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW4" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AX4" s="9"/>
+      <x:c r="AY4" s="9"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="inlineStr">
@@ -1140,6 +1182,18 @@
       <x:c r="AU5" s="8" t="n">
         <x:v>4</x:v>
       </x:c>
+      <x:c r="AV5" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW5" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AX5" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AY5" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="inlineStr">
@@ -1292,6 +1346,18 @@
       </x:c>
       <x:c r="AU6" s="8" t="n">
         <x:v>4</x:v>
+      </x:c>
+      <x:c r="AV6" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AW6" s="9" t="n">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="AX6" s="9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="AY6" s="9" t="n">
+        <x:v>100</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>